<commit_message>
Mise a jour du suivi d'ia Tom BOTTAZZINI
</commit_message>
<xml_diff>
--- a/IA_Tom_BOTTAZZINI.xlsx
+++ b/IA_Tom_BOTTAZZINI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\M2_Progr\m2_2025-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6123913D-9561-4E6D-B64F-3DC6FDB01D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFD1A40-B3C5-438F-A16B-4856F9A75827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2505" yWindow="1965" windowWidth="21600" windowHeight="11295" xr2:uid="{618AA5E7-4921-4257-B0C0-E4DE7D2E073D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{618AA5E7-4921-4257-B0C0-E4DE7D2E073D}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,9 +39,63 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">Date </t>
+  </si>
+  <si>
+    <t>Objectif</t>
+  </si>
+  <si>
+    <t>Promt</t>
+  </si>
+  <si>
+    <t>Résulta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crée la coquie vide du projet </t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Donnée le context a l'IA</t>
+  </si>
+  <si>
+    <t>Commentaire</t>
+  </si>
+  <si>
+    <t>J'ai crée un projet sur Chat GPT et j'ai ajouter dans la partie source le fichier de consigne, et plusieur rappelle en fichier textes</t>
+  </si>
+  <si>
+    <t>Source ajouter</t>
+  </si>
+  <si>
+    <t>Férifier le contexte</t>
+  </si>
+  <si>
+    <t>Fais moi un rappel, du contexte est des consigne, que tu as en sources</t>
+  </si>
+  <si>
+    <t>Résumer des consigne</t>
+  </si>
+  <si>
+    <t>Contexte bien ajouter dans la mémoire du projet</t>
+  </si>
+  <si>
+    <t>tu peux crée, la structure vide, du fichier .py , avec les lib utiles ... mette a jour l'en tête, et ajoute une section consigne ou tu mette le contenue du résumer utra condense # -*- coding: utf-8 -*- """ Éditeur de Spyder Ceci est un script temporaire. Ceci et un fichier de test """ import csv # Chargement dans Python signals_matrix = np.load("signals_matrix.npy")</t>
+  </si>
+  <si>
+    <t>Fichier main.py ; Coqui vide qui lance une fenetre vide</t>
+  </si>
+  <si>
+    <t>je vais faire le fichier READ ME, voici ce que j'avais préparer Nous somme le groupe A, notre objectif est d'Acquérir le signale d'entrée Le fichier d'entrée est de Type CSV. La première colonne le temps, l'instant ou la donnée a étais enregistrais. La deuxième colonne la donnée La Première ligne est une en tête. EXEMPLE: t,x 0.0,4.366025403784439 0.0001220703125,3.6760321842572776 0.000244140625,2.693626153693505 Le fichier de sortie et un fichier CSV: Auteurs : ---------- - Manal BETTAOUI Responsable de l'interface - Alex GRAPIN Responsable de la génération du fichier de sortie - Simon SILVESTRE Responsable de l'extraction des information - Tom BOTTAZZINI Responsable de l'interconnexion et support /// voici les consigne, / Corrige les fautes d'orthographe, et la formulation</t>
+  </si>
+  <si>
+    <t>Mise en form du fichier READ ME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Des piste d'information pour le fichier READ ME, et une correction de l'ortographe </t>
   </si>
 </sst>
 </file>
@@ -77,9 +131,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -414,23 +482,98 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F72C625-8B46-4651-B30B-15F425D4D739}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="48.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="65" style="1" customWidth="1"/>
+    <col min="4" max="4" width="53.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="81" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+    <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>46155</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>46155</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>46155</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="4"/>
+    </row>
+    <row r="5" spans="1:5" ht="180" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>46155</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ajout de deux requettes IA
</commit_message>
<xml_diff>
--- a/IA_Tom_BOTTAZZINI.xlsx
+++ b/IA_Tom_BOTTAZZINI.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\M2_Progr\m2_2025-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFD1A40-B3C5-438F-A16B-4856F9A75827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB3F7981-4C67-4A82-93E7-7363E0F6FC0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{618AA5E7-4921-4257-B0C0-E4DE7D2E073D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">Date </t>
   </si>
@@ -92,10 +92,28 @@
     <t>je vais faire le fichier READ ME, voici ce que j'avais préparer Nous somme le groupe A, notre objectif est d'Acquérir le signale d'entrée Le fichier d'entrée est de Type CSV. La première colonne le temps, l'instant ou la donnée a étais enregistrais. La deuxième colonne la donnée La Première ligne est une en tête. EXEMPLE: t,x 0.0,4.366025403784439 0.0001220703125,3.6760321842572776 0.000244140625,2.693626153693505 Le fichier de sortie et un fichier CSV: Auteurs : ---------- - Manal BETTAOUI Responsable de l'interface - Alex GRAPIN Responsable de la génération du fichier de sortie - Simon SILVESTRE Responsable de l'extraction des information - Tom BOTTAZZINI Responsable de l'interconnexion et support /// voici les consigne, / Corrige les fautes d'orthographe, et la formulation</t>
   </si>
   <si>
-    <t>Mise en form du fichier READ ME</t>
-  </si>
-  <si>
     <t xml:space="preserve">Des piste d'information pour le fichier READ ME, et une correction de l'ortographe </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trouver les paramètre des variable de des module QT </t>
+  </si>
+  <si>
+    <t>je veux écrire dans un Qlabel self.Bulle_taux_echantillon. = mon_signal.sample_rate ;</t>
+  </si>
+  <si>
+    <t>Le bon paramètre, qui permet de l'accées au champs</t>
+  </si>
+  <si>
+    <t>Correction d'une séction du READ ME A</t>
+  </si>
+  <si>
+    <t>Mise en form du fichier READ ME A</t>
+  </si>
+  <si>
+    <t>corrige cet section de text READMEA # Fichier de sortie Le fichier de sortie et un fichier CSV: # Comment utiliser le projet Executer le main.py Ajouter le fichier Cliquer sur le bouton "Fichier" Le lien du fichier s'ajoute dans la zone "Lien" Compléter les informations suivante sur le fichier ajouter: "Type de signal" "Sources" Cliquer ensuite sur "Générer" Vous pouvez observer les paramétres de votre fichier De plus le fichier de sortie est générer "Output_GroupeA.txt"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le paragraphe corriger, </t>
   </si>
 </sst>
 </file>
@@ -482,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F72C625-8B46-4651-B30B-15F425D4D739}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" style="1" customWidth="1"/>
@@ -563,13 +581,41 @@
         <v>46155</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>46183</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>18</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>46189</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Création de la présentation
</commit_message>
<xml_diff>
--- a/IA_Tom_BOTTAZZINI.xlsx
+++ b/IA_Tom_BOTTAZZINI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\M2_Progr\m2_2025-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB3F7981-4C67-4A82-93E7-7363E0F6FC0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4386AE47-6ABE-4F8B-AB01-D6AA37568F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{618AA5E7-4921-4257-B0C0-E4DE7D2E073D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">Date </t>
   </si>
@@ -114,6 +114,15 @@
   </si>
   <si>
     <t xml:space="preserve">Le paragraphe corriger, </t>
+  </si>
+  <si>
+    <t>Création support de présentation</t>
+  </si>
+  <si>
+    <t>La présentation complètet</t>
+  </si>
+  <si>
+    <t>On dois présenter ce projet voici le cahier des charges Présentation de vos travaux Objectifs Présenter votre travail comme si personne ne savait ce que vous faisiez afin de permettre de comprendre : • l’objectif global • le cahier des charges • les choix technologiques (modules, outils, etc) 1 Présentation de votre partie • les choix de programmation réalisés • votre méthodologie de travail • tout autre choses que vous voulez dire ... 1. rappel de votre cahier des charges global et de votre groupe 2. quelles technologies ont été utilisées et pourquoi 3. quels ont été les choix de programmation et pourquoi 4. comment vous vous êtes répartis le travail 5. quelles ont été les points d’appui et les difficultés rencontrées 6. ... 2 Présentation de votre fichier de sortie 1. Quel format de fichier 2. Quels sont les champs du csv (ou du JSON) 3. Si il y a des subtilités (dépendances d’information sur plusieurs lignes par exemple ou si la première ligne est une ligne d’entête, ...) 3 Commentaires Puis enfin toutes les informations supplémentaires que vous aimeriez présenter La présentation doit durer 5 minutes! Voilà, c’est à vous!  prépare pour une présentation génerale, pour le groupe entier # -*- coding: utf-8 -*- """ Projet M2 - Groupe A Module : Acquisition des Signaux Description ----------- Fichier de développement principal du module. Architecture basée sur : - Python 3 - PyQt5 - Pandas - SciPy - Structure modulaire orientée objet (POO) Auteur(s) ---------- - Manal BETTAOUI - Alex GRAPIN - Simon SILVESTRE - Tom BOTTAZZINI Date ----- 2026 Consignes du projet ------------------- Le projet doit respecter les contraintes suivantes : - Application Python modulaire en POO - Utilisation de PyQt5 - Code documenté - Respect des conventions PEP8 et PEP257 - Utilisation de Git pour le versionnement - Architecture propre et maintenable - L’IA doit être utilisée comme assistant technique et non comme générateur complet du projet Technologies obligatoires : - Python v3 uniquement - PyQt5 Designer / pyuic5 - SciPy - Pandas - CSV Bonnes pratiques imposées : - Comprendre le code généré - Tester systématiquement le code - Documenter les fonctions/classes - Éviter le Vibe Coding """ # ============================================================================ # IMPORTS # ============================================================================ import datetime import sys from PyQt5 import QtWidgets from PyQt5.QtWidgets import QFileDialog from Dialog import Ui_Dialog # ============================================================================ # CONSTANTES # ============================================================================ # ============================================================================ # CLASSES # ============================================================================ class MainWindow(Ui_Dialog): """ Fenêtre principale de l'application. """ def __init__(self, dialog): Ui_Dialog.__init__(self) self.setupUi(dialog) self.connexions() def connexions(self): """ La fonction connexions Permet de connecter les signalaux et Slots Paramètres d'entrée : ------- Aucun Returns ------- None Effets ------- Lors d'ppuis dans l'interface on appel des fonctions (slot) """ # Connect the .clicked() signal with the .calculate() slot self.Generer.clicked.connect(self.calculate) # Connexion bouton self.Boutonparcourir.clicked.connect(self.ouvrir_fichier) def calculate(self): """ La fonction calculate Permet de réaliser le coeur du projet. Lors de l'appuis sur le bouton générer cet fonction est appeler Paramètres d'entrée : ------- Aucun Returns ------- None Effets ------- Extrais les donner Appel la fonction de géneration du fichier Réaliser le coeur du projet """ # Nom et localisation du fichier à lire #nom_fichier = "C:\Temp\M2_Progr\m2_2025-2026\Fichier_entree.csv" nom_fichier = self.AffichageURL.text() # On crée un objet "mon_signal" à partir de la classe Mon_Signal_GrpA mon_signal = MonSignalGrpA() # On appelle la méthode d'acquisition (Etape 1) try: mon_signal.acquisition_signal(nom_fichier) except Exception as e: print(f"Erreur : {e}") # On appelle la méthode de traitement (Etape 2) mon_signal.traitement_signal() # A remplir par Manal mon_signal.type = self.comboBox_Type.currentText() mon_signal.source = self.comboBox_Source.currentText() # AFFICHAGE POUR VERIFIER QUE TOUT FONCTIONNE print(" PROPRIÉTÉS DU SIGNAL :") print(f"Type : {mon_signal.type}") print(f"Source : {mon_signal.source}") print(f"Taux d'échantillonnage (sample_rate) : {mon_signal.sample_rate} Hz") self.Affichage_echantillon.setText(f"{mon_signal.sample_rate} Hz") print(f"Durée du signal (duration) : {mon_signal.duration} s") self.Affichage_duree_siganl.setText(f"{mon_signal.duration} s") print(f"Timestamp : {mon_signal.timestamp}") self.Affichage_uptdate.setText(f"{mon_signal.timestamp}") print(f"Nombre d'échantillons : {len(mon_signal.samples)}") self.Affichage_nb_echantillon.setText(f"{len(mon_signal.samples)}") print(f"Aperçu des 5 premiers samples : {mon_signal.samples[:5]}") def ouvrir_fichier(self): """ La fonction ouvrir_fichier Permet d'ouvrir l'exporateur de fichier, pour sélection le fichier d'entrée Un filtre est appliquer pour ouvrire uniquement un fichier .csv Paramètres d'entrée : ------- Aucun Returns ------- None Effets ------- Charge le fichier d'entrée """ file_path, _ = QFileDialog.getOpenFileName( None, "Choisir un fichier", "", "Tous les fichiers (*csv*)" ) if file_path: self.AffichageURL.setText(file_path) class MonSignalGrpA: # Le constructeur : il initialise les variables quand on crée le signal def __init__(self): self.type = "" self.source = "" self.sample_rate = 0 self.duration = 0.0 self.timestamp = "" self.samples = [] # Variable interne du vecteur temps du signal self.t = [] # ETAPE 1 : EXTRACTION DES DONNEES def acquisition_signal(self, filename): """ La fonction Acquisition_signal lit le fichier CSV contenant le signal. Paramètres d'entrée : ------- filename : str (chemin du fichier + nom du fichier) Returns ------- None Effets ------- On remplit les attributs suivants : - self.t : liste des temps - self.samples : liste des échantillons du signal """ # On vide les listes au cas où on réutiliserait la fonction self.t = [] self.samples = [] with open(filename, "r") as f: next(f) # saute la première ligne (les en-têtes) for ligne in f: ligne = ligne.strip() #enlever les espaces et retours à la ligne if not ligne: # Sécurité : ignorer les lignes vides continue valeurs = ligne.split(",") # Le séparateur est une virgule # On stocke les données dans les attributs de la classe (self) self.t.append(float(valeurs[0])) self.samples.append(float(valeurs[1])) # ETAPE 2 : TRAITEMENT DES DONNEES POUR CALCULER LES INFORMATIONS DU SIGNAL def traitement_signal(self): """ La fonction Traitement_signal traite le signal. Paramètres d'entrée : ------- Aucun Returns ------- None Effets ------- On remplit les attributs suivants : - self.sample_rate : Fréquence du signal - self.duration : Durée du signal - self.timestamp : Date de traitement du signal """ # On s'assure qu'il y a au moins 2 points de mesures pour pouvoir faire des calculs if len(self.t) &gt;= 2: # Taux d'échantillonnage (en Hz) dt = self.t[1] - self.t[0] # Période d'échantillonnage self.sample_rate = round(1.0 / dt) # 1 / dt donne la fréquence. "round()" arrondit à l'entier # Durée du signal (en secondes) self.duration = self.t[-1] - self.t[0] # t[-1] permet de récupérer le dernier élément else: self.sample_rate = 0 self.duration = 0 # Timestamp (Horodatage de l'extraction) # datetime.now() récupère la date/heure du PC # .replace(microsecond=0) pour ne pas afficher les microsecondes # .isoformat() formate les données au format iso (ex: 2026-05-13T15:55:00) self.timestamp = datetime.datetime.now().replace(microsecond=0).isoformat() # ============================================================================ # FONCTIONS # ============================================================================ # ============================================================================ # MAIN # ============================================================================ if __name__ == "__main__": app = QtWidgets.QApplication(sys.argv) Dialog = QtWidgets.QDialog() ui = MainWindow(Dialog) Dialog.show() sys.exit(app.exec_()) tu as le code pour complètet et l'interface graphique : # -*- coding: utf-8 -*- # Form implementation generated from reading ui file 'Dialog.ui' # # Created by: PyQt5 UI code generator 5.15.10 # # WARNING: Any manual changes made to this file will be lost when pyuic5 is # run again. Do not edit this file unless you know what you are doing. from PyQt5 import QtCore, QtGui, QtWidgets class Ui_Dialog(object): def setupUi(self, Dialog): Dialog.setObjectName("Dialog") Dialog.resize(689, 460) self.Bullenom = QtWidgets.QTextBrowser(Dialog) self.Bullenom.setGeometry(QtCore.QRect(10, 380, 281, 51)) self.Bullenom.setObjectName("Bullenom") self.BulleTitre = QtWidgets.QTextBrowser(Dialog) self.BulleTitre.setGeometry(QtCore.QRect(10, 10, 281, 51)) self.BulleTitre.setObjectName("BulleTitre") self.AffichageURL = QtWidgets.QLineEdit(Dialog) self.AffichageURL.setGeometry(QtCore.QRect(40, 90, 511, 20)) self.AffichageURL.setObjectName("AffichageURL") self.Boutonparcourir = QtWidgets.QPushButton(Dialog) self.Boutonparcourir.setGeometry(QtCore.QRect(560, 90, 41, 21)) self.Boutonparcourir.setObjectName("Boutonparcourir") self.Lien = QtWidgets.QLabel(Dialog) self.Lien.setGeometry(QtCore.QRect(20, 70, 47, 13)) self.Lien.setObjectName("Lien") self.Type = QtWidgets.QLabel(Dialog) self.Type.setGeometry(QtCore.QRect(10, 130, 91, 16)) self.Type.setObjectName("Type") self.Source = QtWidgets.QLabel(Dialog) self.Source.setGeometry(QtCore.QRect(10, 180, 47, 13)) self.Source.setObjectName("Source") self.comboBox_Type = QtWidgets.QComboBox(Dialog) self.comboBox_Type.setGeometry(QtCore.QRect(50, 150, 181, 22)) self.comboBox_Type.setObjectName("comboBox_Type") self.comboBox_Type.addItem("") self.comboBox_Type.addItem("") self.comboBox_Type.addItem("") self.comboBox_Type.addItem("") self.comboBox_Source = QtWidgets.QComboBox(Dialog) self.comboBox_Source.setGeometry(QtCore.QRect(50, 200, 181, 22)) self.comboBox_Source.setObjectName("comboBox_Source") self.comboBox_Source.addItem("") self.comboBox_Source.addItem("") self.comboBox_Source.addItem("") self.comboBox_Source.addItem("") self.comboBox_Source.addItem("") self.Exit = QtWidgets.QPushButton(Dialog) self.Exit.setGeometry(QtCore.QRect(580, 400, 75, 23)) self.Exit.setObjectName("Exit") self.Generer = QtWidgets.QPushButton(Dialog) self.Generer.setGeometry(QtCore.QRect(580, 360, 75, 23)) self.Generer.setObjectName("Generer") self.Bulle_taux_echantillon = QtWidgets.QLabel(Dialog) self.Bulle_taux_echantillon.setGeometry(QtCore.QRect(350, 140, 131, 21)) self.Bulle_taux_echantillon.setObjectName("Bulle_taux_echantillon") self.Affichage_echantillon = QtWidgets.QLabel(Dialog) self.Affichage_echantillon.setGeometry(QtCore.QRect(480, 140, 61, 20)) self.Affichage_echantillon.setText("") self.Affichage_echantillon.setObjectName("Affichage_echantillon") self.Bulle_enregistrement = QtWidgets.QLabel(Dialog) self.Bulle_enregistrement.setGeometry(QtCore.QRect(350, 170, 131, 21)) self.Bulle_enregistrement.setObjectName("Bulle_enregistrement") self.Affichage_uptdate = QtWidgets.QLabel(Dialog) self.Affichage_uptdate.setGeometry(QtCore.QRect(490, 170, 61, 20)) self.Affichage_uptdate.setText("") self.Affichage_uptdate.setObjectName("Affichage_uptdate") self.Affichage_nb_echantillon = QtWidgets.QLabel(Dialog) self.Affichage_nb_echantillon.setGeometry(QtCore.QRect(480, 200, 61, 20)) self.Affichage_nb_echantillon.setText("") self.Affichage_nb_echantillon.setObjectName("Affichage_nb_echantillon") self.Bulle_nb_echantillon = QtWidgets.QLabel(Dialog) self.Bulle_nb_echantillon.setGeometry(QtCore.QRect(350, 200, 131, 21)) self.Bulle_nb_echantillon.setObjectName("Bulle_nb_echantillon") self.Bulle_duree_du_signal = QtWidgets.QLabel(Dialog) self.Bulle_duree_du_signal.setGeometry(QtCore.QRect(350, 230, 131, 21)) self.Bulle_duree_du_signal.setObjectName("Bulle_duree_du_signal") self.Affichage_duree_siganl = QtWidgets.QLabel(Dialog) self.Affichage_duree_siganl.setGeometry(QtCore.QRect(480, 230, 61, 20)) self.Affichage_duree_siganl.setText("") self.Affichage_duree_siganl.setObjectName("Affichage_duree_siganl") self.retranslateUi(Dialog) QtCore.QMetaObject.connectSlotsByName(Dialog) def retranslateUi(self, Dialog): _translate = QtCore.QCoreApplication.translate Dialog.setWindowTitle(_translate("Dialog", "Dialog")) self.Bullenom.setHtml(_translate("Dialog", "&lt;!DOCTYPE HTML PUBLIC \"-//W3C//DTD HTML 4.0//EN\" \"http://www.w3.org/TR/REC-html40/strict.dtd\"&gt;\n" "&lt;html&gt;&lt;head&gt;&lt;meta name=\"qrichtext\" content=\"1\" /&gt;&lt;style type=\"text/css\"&gt;\n" "p, li { white-space: pre-wrap; }\n" "&lt;/style&gt;&lt;/head&gt;&lt;body style=\" font-family:\'MS Shell Dlg 2\'; font-size:8.25pt; font-weight:400; font-style:normal;\"&gt;\n" "&lt;p style=\" margin-top:0px; margin-bottom:0px; margin-left:0px; margin-right:0px; -qt-block-indent:0; text-indent:0px;\"&gt;&lt;span style=\" font-size:8pt; font-weight:600; color:#ffaa00;\"&gt;Classe : M2-3EA&lt;/span&gt;&lt;/p&gt;\n" "&lt;p style=\" margin-top:0px; margin-bottom:0px; margin-left:0px; margin-right:0px; -qt-block-indent:0; text-indent:0px;\"&gt;&lt;span style=\" font-size:8pt; font-weight:600; color:#000000;\"&gt;Groupe : &lt;/span&gt;&lt;/p&gt;\n" "&lt;p style=\" margin-top:0px; margin-bottom:0px; margin-left:0px; margin-right:0px; -qt-block-indent:0; text-indent:0px;\"&gt;&lt;span style=\" font-size:8pt; font-weight:600; color:#000000;\"&gt;BOTTAZZINI ; BETTAOUI ; SILVESTRE ; GRAPIN&lt;/span&gt;&lt;/p&gt;&lt;/body&gt;&lt;/html&gt;")) self.BulleTitre.setHtml(_translate("Dialog", "&lt;!DOCTYPE HTML PUBLIC \"-//W3C//DTD HTML 4.0//EN\" \"http://www.w3.org/TR/REC-html40/strict.dtd\"&gt;\n" "&lt;html&gt;&lt;head&gt;&lt;meta name=\"qrichtext\" content=\"1\" /&gt;&lt;style type=\"text/css\"&gt;\n" "p, li { white-space: pre-wrap; }\n" "&lt;/style&gt;&lt;/head&gt;&lt;body style=\" font-family:\'MS Shell Dlg 2\'; font-size:8.25pt; font-weight:400; font-style:normal;\"&gt;\n" "&lt;p style=\" margin-top:0px; margin-bottom:0px; margin-left:0px; margin-right:0px; -qt-block-indent:0; text-indent:0px;\"&gt;&lt;span style=\" font-size:16pt; font-weight:600; color:#ffaa00;\"&gt;Traitement de signal&lt;/span&gt;&lt;/p&gt;\n" "&lt;p style=\" margin-top:0px; margin-bottom:0px; margin-left:0px; margin-right:0px; -qt-block-indent:0; text-indent:0px;\"&gt;&lt;span style=\" font-size:9pt; font-weight:600; color:#000000;\"&gt;Partie A : Acquisition du signal&lt;/span&gt;&lt;/p&gt;&lt;/body&gt;&lt;/html&gt;")) self.Boutonparcourir.setText(_translate("Dialog", "...")) self.Lien.setText(_translate("Dialog", "Lien :")) self.Type.setText(_translate("Dialog", "Type de Signal :")) self.Source.setText(_translate("Dialog", "Sources :")) self.comboBox_Type.setItemText(0, _translate("Dialog", "Entrer Texte")) self.comboBox_Type.setItemText(1, _translate("Dialog", "Audio")) self.comboBox_Type.setItemText(2, _translate("Dialog", "Vidéo")) self.comboBox_Type.setItemText(3, _translate("Dialog", "Image")) self.comboBox_Source.setItemText(0, _translate("Dialog", "Entrer Texte")) self.comboBox_Source.setItemText(1, _translate("Dialog", "Microphone")) self.comboBox_Source.setItemText(2, _translate("Dialog", "Capteurs")) self.comboBox_Source.setItemText(3, _translate("Dialog", "Caméra")) self.comboBox_Source.setItemText(4, _translate("Dialog", "Fichier")) self.Exit.setText(_translate("Dialog", "Exit")) self.Generer.setText(_translate("Dialog", "Générer")) self.Bulle_taux_echantillon.setText(_translate("Dialog", "Taux d\'échantillonage : ")) self.Bulle_enregistrement.setText(_translate("Dialog", "Derniere enregistrement :")) self.Bulle_nb_echantillon.setText(_translate("Dialog", "Nombre d\'échantillon : ")) self.Bulle_duree_du_signal.setText(_translate("Dialog", "Durée du signal"))</t>
   </si>
 </sst>
 </file>
@@ -149,22 +158,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -500,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F72C625-8B46-4651-B30B-15F425D4D739}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" style="1" customWidth="1"/>
@@ -511,112 +514,130 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>46155</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>46155</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="92.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+      <c r="A4" s="3">
         <v>46155</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="4"/>
+      <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:5" ht="180" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+      <c r="A5" s="3">
         <v>46155</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>17</v>
       </c>
+      <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="A6" s="3">
         <v>46183</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="105" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="A7" s="3">
         <v>46189</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>46190</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>